<commit_message>
feat(reporting): standardize objective model input
Context
Goal: 将 model_input_metrics.csv 收敛为稳定的客观指标、来源、覆盖率和质量说明接口。
Reason: 阶段 5 要防止仓库输出投资建议、颜色状态、方向判断或买卖动作，并完成既定八列模型输入契约。

Changes
Updated: model input builder 固定输出 metric_name、metric_value、metric_date、source、provider、coverage_ratio、is_missing、quality_message。
Updated: 价格、宏观、广度和 data quality 指标按数据集来源与 provider 分离映射，覆盖率仅写入覆盖类指标。
Added: 禁用词、旧输出文件名、manifest 索引和字段映射防回归测试。
Updated: README、数据模型文档和 ChatGPT 示例说明新版客观字段契约。
Captured: 重新生成 2026-06-06 model_input_metrics、manifest、Excel 和相关 daily 报告。

State
Compile/Test: Passed - uv run pytest (40 passed); uv run python scripts/run_daily.py --as-of auto
Side Effects: 未生成 analysis_summary.* 或 ai_input.csv；twelvedata_api_test_pack.zip 保持未跟踪，未纳入提交。

Next
完整优化计划阶段 1-5 已落地，可继续独立规划 manual cache rebuild 或 weekly cache audit。
</commit_message>
<xml_diff>
--- a/reports/archive/2026-06-06/nasdaq100_qqq_daily_tracker_2026-06-06.xlsx
+++ b/reports/archive/2026-06-06/nasdaq100_qqq_daily_tracker_2026-06-06.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">宏观指标!$A$1:$E$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">市场广度!$A$1:$F$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">数据质量!$A$1:$O$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">模型输入指标!$A$1:$F$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">模型输入指标!$A$1:$H$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">运行日志!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2533" uniqueCount="549">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2614" uniqueCount="562">
   <si>
     <t>date</t>
   </si>
@@ -1357,6 +1357,9 @@
     <t>NVDA,AAPL,MSFT,MU,AMZN,AMD,GOOGL,TSLA,GOOG,AVGO,META,WMT,INTC,CSCO,COST,LRCX,AMAT,NFLX,PLTR,KLAC,TXN,MRVL,QCOM,SNDK,LIN,PANW,ADI,STX,TMUS,WDC,PEP,AMGN,CRWD,APP,GILD,ISRG,SHOP,HON,BKNG,CDNS,VRTX,FTNT,SBUX,ADBE,MAR,CEG,SNPS,ADP,MNST,CSX,CMCSA,INTU,MELI,NXPI,MPWR,DDOG,MDLZ,ROST,ORLY,CTAS,AEP,LITE,WBD,DASH,BKR,REGN,PCAR,FANG,ABNB,FAST,MCHP,ODFL,EA,ADSK,XEL,FER,EXC,IDXX,CCEP,AXON,KDP,MSTR,ALNY,TTWO,PYPL,TRI,PAYX,ROP,WDAY,CPRT,GEHC,DXCM,KHC,CTSH,VRSK,INSM,ZS,CHTR</t>
   </si>
   <si>
+    <t>GOOG,AVGO</t>
+  </si>
+  <si>
     <t>ADI,ALNY,AMAT,AMD,AMZN,AVGO,AXON,CCEP,CHTR,COST,CPRT,CSCO,CTSH,DXCM,GEHC,GOOG,GOOGL,IDXX,INSM,INTC,KDP,KHC,KLAC,LIN,LRCX,META,MRVL,MSTR,NFLX,PANW,PAYX,PLTR,PYPL,QCOM,ROP,SNDK,STX,TRI,TSLA,TTWO,TXN,VRSK,WDAY,WMT,ZS</t>
   </si>
   <si>
@@ -1399,7 +1402,7 @@
     <t>0/98 quotes fetched</t>
   </si>
   <si>
-    <t>20/20 top20 quotes available; 10/10 top10 quotes available</t>
+    <t>18/20 top20 quotes available; 8/10 top10 quotes available</t>
   </si>
   <si>
     <t>53/98 symbols with history+quote coverage; coverage insufficient for top-weight symbols</t>
@@ -1480,6 +1483,9 @@
     <t>NVDA,AAPL,MSFT,MU,AMZN,AMD,GOOGL,TSLA,GOOG,AVGO,META,WMT,INTC,CSCO,COST,LRCX,AMAT,NFLX,PLTR,KLAC</t>
   </si>
   <si>
+    <t>NVDA,AAPL,MSFT,MU,AMZN,AMD,GOOGL,TSLA,META,WMT,INTC,CSCO,COST,LRCX,AMAT,NFLX,PLTR,KLAC</t>
+  </si>
+  <si>
     <t>DGS10: DGS10: 365 rows; DGS2: DGS2: 365 rows; DGS3MO: DGS3MO: 365 rows; ...</t>
   </si>
   <si>
@@ -1495,6 +1501,15 @@
     <t>provider not called in this daily pipeline run</t>
   </si>
   <si>
+    <t>metric_date</t>
+  </si>
+  <si>
+    <t>coverage_ratio</t>
+  </si>
+  <si>
+    <t>quality_message</t>
+  </si>
+  <si>
     <t>QQQ_latest_close</t>
   </si>
   <si>
@@ -1603,6 +1618,15 @@
     <t>breadth_metrics_fmp+tiingo_cache_rate_limited</t>
   </si>
   <si>
+    <t>price_metrics</t>
+  </si>
+  <si>
+    <t>macro_metrics</t>
+  </si>
+  <si>
+    <t>data_quality</t>
+  </si>
+  <si>
     <t>latest adjusted close</t>
   </si>
   <si>
@@ -1636,40 +1660,55 @@
     <t>breadth metric; denominator=53</t>
   </si>
   <si>
-    <t>data quality symbol coverage; ok=True; rows=100</t>
-  </si>
-  <si>
-    <t>data quality weight coverage; rate_limited=False; fallback_provider=</t>
-  </si>
-  <si>
-    <t>1 means provider hit 429 and breadth stopped_after_429=False</t>
-  </si>
-  <si>
-    <t>data quality symbol coverage; ok=True; rows=365</t>
-  </si>
-  <si>
-    <t>data quality symbol coverage; ok=True; rows=104</t>
-  </si>
-  <si>
-    <t>data quality symbol coverage; ok=True; rows=98</t>
-  </si>
-  <si>
-    <t>data quality symbol coverage; ok=False; rows=98</t>
-  </si>
-  <si>
-    <t>data quality symbol coverage; ok=True; rows=20</t>
-  </si>
-  <si>
-    <t>data quality weight coverage; rate_limited=False; fallback_provider=twelve_data</t>
-  </si>
-  <si>
-    <t>data quality symbol coverage; ok=True; rows=8</t>
-  </si>
-  <si>
-    <t>data quality weight coverage; rate_limited=False; fallback_provider=mixed_fmp+tiingo_history_only</t>
-  </si>
-  <si>
-    <t>FMP</t>
+    <t>symbol coverage; ok=True; rows=100; message=QQQ: 100 rows</t>
+  </si>
+  <si>
+    <t>weight coverage; rate_limited=False; fallback_provider=</t>
+  </si>
+  <si>
+    <t>1 means provider hit a limit; stopped_after_429=False</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=True; rows=365; message=DGS10: 365 rows</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=True; rows=365; message=DGS2: 365 rows</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=True; rows=365; message=DGS3MO: 365 rows</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=True; rows=365; message=DFF: 365 rows</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=True; rows=365; message=CPIAUCSL: 365 rows</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=True; rows=365; message=PCEPI: 365 rows</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=True; rows=365; message=UNRATE: 365 rows</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=True; rows=104; message=QQQ: holdings rows=104 effective_date=2026-06-04</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=True; rows=98; message=equity filter applied for breadth stock pool</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=False; rows=98; message=0/98 quotes fetched</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=True; rows=20; message=18/20 top20 quotes available; 8/10 top10 quotes available</t>
+  </si>
+  <si>
+    <t>weight coverage; rate_limited=False; fallback_provider=twelve_data</t>
+  </si>
+  <si>
+    <t>symbol coverage; ok=True; rows=8; message=53/98 symbols with history+quote coverage; coverage insufficient for top-weight symbols</t>
+  </si>
+  <si>
+    <t>weight coverage; rate_limited=False; fallback_provider=mixed_fmp+tiingo_history_only</t>
   </si>
   <si>
     <t>method</t>
@@ -5019,46 +5058,46 @@
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="2" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>408</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>418</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>419</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>424</v>
@@ -5066,13 +5105,13 @@
     </row>
     <row r="2" spans="1:15">
       <c r="A2" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B2" t="s">
         <v>110</v>
       </c>
       <c r="C2" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -5087,7 +5126,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="I2">
         <v>25</v>
@@ -5105,18 +5144,18 @@
         <v>0</v>
       </c>
       <c r="O2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="3" spans="1:15">
       <c r="A3" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B3" t="s">
         <v>432</v>
       </c>
       <c r="C3" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D3">
         <v>7</v>
@@ -5131,7 +5170,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="I3">
         <v>10</v>
@@ -5140,21 +5179,21 @@
         <v>7</v>
       </c>
       <c r="K3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="L3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="M3" t="b">
         <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="4" spans="1:15">
       <c r="A4" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B4" t="s">
         <v>390</v>
@@ -5175,7 +5214,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="I4">
         <v>3</v>
@@ -5193,18 +5232,18 @@
         <v>0</v>
       </c>
       <c r="O4" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B5" t="s">
         <v>434</v>
       </c>
       <c r="C5" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -5219,7 +5258,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="I5">
         <v>250</v>
@@ -5228,39 +5267,39 @@
         <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="M5" t="b">
         <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B6" t="s">
         <v>410</v>
       </c>
       <c r="C6" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D6">
         <v>20</v>
       </c>
       <c r="E6">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" t="b">
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="I6">
         <v>8</v>
@@ -5269,27 +5308,27 @@
         <v>20</v>
       </c>
       <c r="K6" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="L6" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="M6" t="b">
         <v>0</v>
       </c>
       <c r="O6" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B7" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C7" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -5304,7 +5343,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="I7">
         <v>50</v>
@@ -5316,7 +5355,7 @@
         <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>
@@ -5358,7 +5397,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -5372,7 +5411,7 @@
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -5386,7 +5425,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -5400,7 +5439,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -5414,7 +5453,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -5428,7 +5467,7 @@
         <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -5442,7 +5481,7 @@
         <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -5456,7 +5495,7 @@
         <v>0</v>
       </c>
       <c r="D9" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -5470,7 +5509,7 @@
         <v>0</v>
       </c>
       <c r="D10" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -5484,7 +5523,7 @@
         <v>0</v>
       </c>
       <c r="D11" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -5498,7 +5537,7 @@
         <v>0</v>
       </c>
       <c r="D12" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -5512,7 +5551,7 @@
         <v>0</v>
       </c>
       <c r="D13" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -5526,7 +5565,7 @@
         <v>0</v>
       </c>
       <c r="D14" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -5540,7 +5579,7 @@
         <v>0</v>
       </c>
       <c r="D15" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -5554,7 +5593,7 @@
         <v>0</v>
       </c>
       <c r="D16" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -5568,7 +5607,7 @@
         <v>0</v>
       </c>
       <c r="D17" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -5582,7 +5621,7 @@
         <v>0</v>
       </c>
       <c r="D18" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -5596,7 +5635,7 @@
         <v>0</v>
       </c>
       <c r="D19" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -5610,7 +5649,7 @@
         <v>0</v>
       </c>
       <c r="D20" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -5624,7 +5663,7 @@
         <v>0</v>
       </c>
       <c r="D21" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -5638,7 +5677,7 @@
         <v>0</v>
       </c>
       <c r="D22" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -5652,7 +5691,7 @@
         <v>0</v>
       </c>
       <c r="D23" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -5666,7 +5705,7 @@
         <v>0</v>
       </c>
       <c r="D24" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -5680,7 +5719,7 @@
         <v>0</v>
       </c>
       <c r="D25" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -5694,7 +5733,7 @@
         <v>0</v>
       </c>
       <c r="D26" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -5708,7 +5747,7 @@
         <v>0</v>
       </c>
       <c r="D27" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -5722,7 +5761,7 @@
         <v>0</v>
       </c>
       <c r="D28" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -5736,7 +5775,7 @@
         <v>0</v>
       </c>
       <c r="D29" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -5750,7 +5789,7 @@
         <v>0</v>
       </c>
       <c r="D30" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -5764,7 +5803,7 @@
         <v>0</v>
       </c>
       <c r="D31" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -5778,7 +5817,7 @@
         <v>0</v>
       </c>
       <c r="D32" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -5792,7 +5831,7 @@
         <v>0</v>
       </c>
       <c r="D33" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -5806,7 +5845,7 @@
         <v>0</v>
       </c>
       <c r="D34" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -5820,7 +5859,7 @@
         <v>0</v>
       </c>
       <c r="D35" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -5834,7 +5873,7 @@
         <v>0</v>
       </c>
       <c r="D36" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -5848,7 +5887,7 @@
         <v>0</v>
       </c>
       <c r="D37" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -5862,7 +5901,7 @@
         <v>0</v>
       </c>
       <c r="D38" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -5876,7 +5915,7 @@
         <v>0</v>
       </c>
       <c r="D39" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -5890,7 +5929,7 @@
         <v>0</v>
       </c>
       <c r="D40" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -5904,7 +5943,7 @@
         <v>0</v>
       </c>
       <c r="D41" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -5918,7 +5957,7 @@
         <v>0</v>
       </c>
       <c r="D42" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -5932,7 +5971,7 @@
         <v>0</v>
       </c>
       <c r="D43" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -5946,7 +5985,7 @@
         <v>0</v>
       </c>
       <c r="D44" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -5960,7 +5999,7 @@
         <v>0</v>
       </c>
       <c r="D45" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -5974,7 +6013,7 @@
         <v>0</v>
       </c>
       <c r="D46" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -5988,7 +6027,7 @@
         <v>0</v>
       </c>
       <c r="D47" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -6002,7 +6041,7 @@
         <v>0</v>
       </c>
       <c r="D48" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -6016,7 +6055,7 @@
         <v>0</v>
       </c>
       <c r="D49" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -6030,7 +6069,7 @@
         <v>0</v>
       </c>
       <c r="D50" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -6044,7 +6083,7 @@
         <v>0</v>
       </c>
       <c r="D51" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -6058,7 +6097,7 @@
         <v>0</v>
       </c>
       <c r="D52" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -6072,7 +6111,7 @@
         <v>0</v>
       </c>
       <c r="D53" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -6086,7 +6125,7 @@
         <v>0</v>
       </c>
       <c r="D54" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -6100,7 +6139,7 @@
         <v>0</v>
       </c>
       <c r="D55" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -6114,7 +6153,7 @@
         <v>0</v>
       </c>
       <c r="D56" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -6128,7 +6167,7 @@
         <v>0</v>
       </c>
       <c r="D57" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -6142,7 +6181,7 @@
         <v>0</v>
       </c>
       <c r="D58" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -6156,7 +6195,7 @@
         <v>0</v>
       </c>
       <c r="D59" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -6170,7 +6209,7 @@
         <v>0</v>
       </c>
       <c r="D60" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -6184,7 +6223,7 @@
         <v>0</v>
       </c>
       <c r="D61" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -6198,7 +6237,7 @@
         <v>0</v>
       </c>
       <c r="D62" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -6212,7 +6251,7 @@
         <v>0</v>
       </c>
       <c r="D63" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -6226,7 +6265,7 @@
         <v>0</v>
       </c>
       <c r="D64" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -6240,7 +6279,7 @@
         <v>0</v>
       </c>
       <c r="D65" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -6254,7 +6293,7 @@
         <v>0</v>
       </c>
       <c r="D66" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -6268,7 +6307,7 @@
         <v>0</v>
       </c>
       <c r="D67" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -6282,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="D68" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -6296,7 +6335,7 @@
         <v>0</v>
       </c>
       <c r="D69" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -6310,7 +6349,7 @@
         <v>0</v>
       </c>
       <c r="D70" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -6324,7 +6363,7 @@
         <v>0</v>
       </c>
       <c r="D71" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -6338,7 +6377,7 @@
         <v>0</v>
       </c>
       <c r="D72" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -6352,7 +6391,7 @@
         <v>0</v>
       </c>
       <c r="D73" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -6366,7 +6405,7 @@
         <v>0</v>
       </c>
       <c r="D74" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -6380,7 +6419,7 @@
         <v>0</v>
       </c>
       <c r="D75" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -6394,7 +6433,7 @@
         <v>0</v>
       </c>
       <c r="D76" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -6408,7 +6447,7 @@
         <v>0</v>
       </c>
       <c r="D77" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -6422,7 +6461,7 @@
         <v>0</v>
       </c>
       <c r="D78" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -6436,7 +6475,7 @@
         <v>0</v>
       </c>
       <c r="D79" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -6450,7 +6489,7 @@
         <v>0</v>
       </c>
       <c r="D80" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -6464,7 +6503,7 @@
         <v>0</v>
       </c>
       <c r="D81" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -6478,7 +6517,7 @@
         <v>0</v>
       </c>
       <c r="D82" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -6492,7 +6531,7 @@
         <v>0</v>
       </c>
       <c r="D83" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -6506,7 +6545,7 @@
         <v>0</v>
       </c>
       <c r="D84" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -6520,7 +6559,7 @@
         <v>0</v>
       </c>
       <c r="D85" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -6534,7 +6573,7 @@
         <v>0</v>
       </c>
       <c r="D86" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -6548,7 +6587,7 @@
         <v>0</v>
       </c>
       <c r="D87" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -6562,7 +6601,7 @@
         <v>0</v>
       </c>
       <c r="D88" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -6576,7 +6615,7 @@
         <v>0</v>
       </c>
       <c r="D89" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -6590,7 +6629,7 @@
         <v>0</v>
       </c>
       <c r="D90" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -6604,7 +6643,7 @@
         <v>0</v>
       </c>
       <c r="D91" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -6618,7 +6657,7 @@
         <v>0</v>
       </c>
       <c r="D92" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -6632,7 +6671,7 @@
         <v>0</v>
       </c>
       <c r="D93" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -6646,7 +6685,7 @@
         <v>0</v>
       </c>
       <c r="D94" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -6660,7 +6699,7 @@
         <v>0</v>
       </c>
       <c r="D95" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -6674,7 +6713,7 @@
         <v>0</v>
       </c>
       <c r="D96" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -6688,7 +6727,7 @@
         <v>0</v>
       </c>
       <c r="D97" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -6702,7 +6741,7 @@
         <v>0</v>
       </c>
       <c r="D98" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -6716,7 +6755,7 @@
         <v>0</v>
       </c>
       <c r="D99" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
   </sheetData>
@@ -6727,18 +6766,19 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" customWidth="1"/>
+    <col min="8" max="8" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8">
       <c r="A1" s="2" t="s">
         <v>138</v>
       </c>
@@ -6746,176 +6786,206 @@
         <v>139</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>140</v>
+        <v>486</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>141</v>
+        <v>8</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>8</v>
+        <v>408</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>392</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="H1" s="2" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
       <c r="B2">
         <v>705.0599999999999</v>
       </c>
       <c r="C2" t="s">
-        <v>520</v>
+        <v>108</v>
       </c>
       <c r="D2" t="s">
-        <v>108</v>
+        <v>525</v>
       </c>
       <c r="E2" t="s">
         <v>110</v>
       </c>
-      <c r="F2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B3">
         <v>0.01456240826546162</v>
       </c>
       <c r="C3" t="s">
-        <v>521</v>
+        <v>108</v>
       </c>
       <c r="D3" t="s">
-        <v>108</v>
+        <v>525</v>
       </c>
       <c r="E3" t="s">
         <v>110</v>
       </c>
-      <c r="F3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="B4">
         <v>0.1602297223913507</v>
       </c>
       <c r="C4" t="s">
-        <v>522</v>
+        <v>108</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>525</v>
       </c>
       <c r="E4" t="s">
         <v>110</v>
       </c>
-      <c r="F4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="B5">
         <v>0.2346381697618982</v>
       </c>
       <c r="C5" t="s">
-        <v>523</v>
+        <v>108</v>
       </c>
       <c r="D5" t="s">
-        <v>108</v>
+        <v>525</v>
       </c>
       <c r="E5" t="s">
         <v>110</v>
       </c>
-      <c r="F5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="B6">
         <v>-0.0550820199421036</v>
       </c>
       <c r="C6" t="s">
-        <v>524</v>
+        <v>108</v>
       </c>
       <c r="D6" t="s">
-        <v>108</v>
+        <v>525</v>
       </c>
       <c r="E6" t="s">
         <v>110</v>
       </c>
-      <c r="F6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="B7">
         <v>-0.1183474937620417</v>
       </c>
       <c r="C7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D7" t="s">
         <v>525</v>
-      </c>
-      <c r="D7" t="s">
-        <v>108</v>
       </c>
       <c r="E7" t="s">
         <v>110</v>
       </c>
-      <c r="F7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B8">
         <v>667.8092</v>
       </c>
       <c r="C8" t="s">
-        <v>526</v>
+        <v>108</v>
       </c>
       <c r="D8" t="s">
-        <v>108</v>
+        <v>525</v>
       </c>
       <c r="E8" t="s">
         <v>110</v>
       </c>
-      <c r="F8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="C9" t="s">
-        <v>527</v>
+        <v>108</v>
       </c>
       <c r="D9" t="s">
-        <v>108</v>
+        <v>525</v>
       </c>
       <c r="E9" t="s">
         <v>110</v>
       </c>
-      <c r="F9" t="b">
+      <c r="G9" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="H9" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>142</v>
       </c>
@@ -6923,139 +6993,160 @@
         <v>4.47</v>
       </c>
       <c r="C10" t="s">
-        <v>528</v>
+        <v>107</v>
       </c>
       <c r="D10" t="s">
-        <v>107</v>
+        <v>426</v>
       </c>
       <c r="E10" t="s">
         <v>137</v>
       </c>
-      <c r="F10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="B11">
         <v>4.05</v>
       </c>
       <c r="C11" t="s">
-        <v>528</v>
+        <v>107</v>
       </c>
       <c r="D11" t="s">
-        <v>107</v>
+        <v>426</v>
       </c>
       <c r="E11" t="s">
         <v>137</v>
       </c>
-      <c r="F11" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="B12">
         <v>3.78</v>
       </c>
       <c r="C12" t="s">
-        <v>528</v>
+        <v>107</v>
       </c>
       <c r="D12" t="s">
-        <v>107</v>
+        <v>426</v>
       </c>
       <c r="E12" t="s">
         <v>137</v>
       </c>
-      <c r="F12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="B13">
         <v>3.62</v>
       </c>
       <c r="C13" t="s">
-        <v>528</v>
+        <v>107</v>
       </c>
       <c r="D13" t="s">
-        <v>107</v>
+        <v>426</v>
       </c>
       <c r="E13" t="s">
         <v>137</v>
       </c>
-      <c r="F13" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
+      <c r="G13" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="B14">
         <v>332.407</v>
       </c>
       <c r="C14" t="s">
-        <v>528</v>
+        <v>63</v>
       </c>
       <c r="D14" t="s">
-        <v>63</v>
+        <v>426</v>
       </c>
       <c r="E14" t="s">
         <v>137</v>
       </c>
-      <c r="F14" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
+      <c r="H14" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="B15">
         <v>130.902</v>
       </c>
       <c r="C15" t="s">
-        <v>528</v>
+        <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>63</v>
+        <v>426</v>
       </c>
       <c r="E15" t="s">
         <v>137</v>
       </c>
-      <c r="F15" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
+      <c r="G15" t="b">
+        <v>0</v>
+      </c>
+      <c r="H15" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="B16">
         <v>4.3</v>
       </c>
       <c r="C16" t="s">
-        <v>528</v>
+        <v>84</v>
       </c>
       <c r="D16" t="s">
-        <v>84</v>
+        <v>426</v>
       </c>
       <c r="E16" t="s">
         <v>137</v>
       </c>
-      <c r="F16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
+      <c r="G16" t="b">
+        <v>0</v>
+      </c>
+      <c r="H16" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" t="s">
         <v>142</v>
       </c>
@@ -7063,19 +7154,22 @@
         <v>4.47</v>
       </c>
       <c r="C17" t="s">
-        <v>156</v>
+        <v>107</v>
       </c>
       <c r="D17" t="s">
-        <v>107</v>
+        <v>526</v>
       </c>
       <c r="E17" t="s">
         <v>137</v>
       </c>
-      <c r="F17" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
+      <c r="G17" t="b">
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" t="s">
         <v>143</v>
       </c>
@@ -7083,19 +7177,22 @@
         <v>0.04000000000000004</v>
       </c>
       <c r="C18" t="s">
-        <v>157</v>
+        <v>107</v>
       </c>
       <c r="D18" t="s">
-        <v>107</v>
+        <v>526</v>
       </c>
       <c r="E18" t="s">
         <v>137</v>
       </c>
-      <c r="F18" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
+      <c r="G18" t="b">
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" t="s">
         <v>144</v>
       </c>
@@ -7103,19 +7200,22 @@
         <v>-0.4199999999999999</v>
       </c>
       <c r="C19" t="s">
-        <v>158</v>
+        <v>107</v>
       </c>
       <c r="D19" t="s">
-        <v>107</v>
+        <v>526</v>
       </c>
       <c r="E19" t="s">
         <v>137</v>
       </c>
-      <c r="F19" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
+      <c r="G19" t="b">
+        <v>0</v>
+      </c>
+      <c r="H19" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" t="s">
         <v>145</v>
       </c>
@@ -7123,19 +7223,22 @@
         <v>0.4199999999999999</v>
       </c>
       <c r="C20" t="s">
-        <v>159</v>
+        <v>107</v>
       </c>
       <c r="D20" t="s">
-        <v>107</v>
+        <v>526</v>
       </c>
       <c r="E20" t="s">
         <v>137</v>
       </c>
-      <c r="F20" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
+      <c r="G20" t="b">
+        <v>0</v>
+      </c>
+      <c r="H20" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" t="s">
         <v>146</v>
       </c>
@@ -7143,19 +7246,22 @@
         <v>-0.07999999999999963</v>
       </c>
       <c r="C21" t="s">
-        <v>160</v>
+        <v>107</v>
       </c>
       <c r="D21" t="s">
-        <v>107</v>
+        <v>526</v>
       </c>
       <c r="E21" t="s">
         <v>137</v>
       </c>
-      <c r="F21" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
+      <c r="G21" t="b">
+        <v>0</v>
+      </c>
+      <c r="H21" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" t="s">
         <v>147</v>
       </c>
@@ -7163,19 +7269,22 @@
         <v>0.00267003074209704</v>
       </c>
       <c r="C22" t="s">
-        <v>161</v>
+        <v>63</v>
       </c>
       <c r="D22" t="s">
-        <v>63</v>
+        <v>526</v>
       </c>
       <c r="E22" t="s">
         <v>137</v>
       </c>
-      <c r="F22" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
+      <c r="G22" t="b">
+        <v>0</v>
+      </c>
+      <c r="H22" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" t="s">
         <v>148</v>
       </c>
@@ -7183,19 +7292,22 @@
         <v>0.008651438343614481</v>
       </c>
       <c r="C23" t="s">
-        <v>161</v>
+        <v>63</v>
       </c>
       <c r="D23" t="s">
-        <v>63</v>
+        <v>526</v>
       </c>
       <c r="E23" t="s">
         <v>137</v>
       </c>
-      <c r="F23" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
+      <c r="G23" t="b">
+        <v>0</v>
+      </c>
+      <c r="H23" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" t="s">
         <v>149</v>
       </c>
@@ -7203,19 +7315,22 @@
         <v>0.006400377846336402</v>
       </c>
       <c r="C24" t="s">
-        <v>161</v>
+        <v>63</v>
       </c>
       <c r="D24" t="s">
-        <v>63</v>
+        <v>526</v>
       </c>
       <c r="E24" t="s">
         <v>137</v>
       </c>
-      <c r="F24" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
+      <c r="G24" t="b">
+        <v>0</v>
+      </c>
+      <c r="H24" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" t="s">
         <v>150</v>
       </c>
@@ -7223,19 +7338,22 @@
         <v>0.006400377846336402</v>
       </c>
       <c r="C25" t="s">
-        <v>162</v>
+        <v>63</v>
       </c>
       <c r="D25" t="s">
-        <v>63</v>
+        <v>526</v>
       </c>
       <c r="E25" t="s">
         <v>137</v>
       </c>
-      <c r="F25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6">
+      <c r="G25" t="b">
+        <v>0</v>
+      </c>
+      <c r="H25" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" t="s">
         <v>151</v>
       </c>
@@ -7243,19 +7361,22 @@
         <v>0.004015441621060045</v>
       </c>
       <c r="C26" t="s">
-        <v>163</v>
+        <v>63</v>
       </c>
       <c r="D26" t="s">
-        <v>63</v>
+        <v>526</v>
       </c>
       <c r="E26" t="s">
         <v>137</v>
       </c>
-      <c r="F26" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6">
+      <c r="G26" t="b">
+        <v>0</v>
+      </c>
+      <c r="H26" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" t="s">
         <v>152</v>
       </c>
@@ -7263,19 +7384,22 @@
         <v>0.006647621988882024</v>
       </c>
       <c r="C27" t="s">
-        <v>163</v>
+        <v>63</v>
       </c>
       <c r="D27" t="s">
-        <v>63</v>
+        <v>526</v>
       </c>
       <c r="E27" t="s">
         <v>137</v>
       </c>
-      <c r="F27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
+      <c r="G27" t="b">
+        <v>0</v>
+      </c>
+      <c r="H27" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28" t="s">
         <v>153</v>
       </c>
@@ -7283,19 +7407,22 @@
         <v>0.003995981009502714</v>
       </c>
       <c r="C28" t="s">
-        <v>163</v>
+        <v>63</v>
       </c>
       <c r="D28" t="s">
-        <v>63</v>
+        <v>526</v>
       </c>
       <c r="E28" t="s">
         <v>137</v>
       </c>
-      <c r="F28" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
+      <c r="G28" t="b">
+        <v>0</v>
+      </c>
+      <c r="H28" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" t="s">
         <v>154</v>
       </c>
@@ -7303,19 +7430,22 @@
         <v>0.003995981009502714</v>
       </c>
       <c r="C29" t="s">
-        <v>164</v>
+        <v>63</v>
       </c>
       <c r="D29" t="s">
-        <v>63</v>
+        <v>526</v>
       </c>
       <c r="E29" t="s">
         <v>137</v>
       </c>
-      <c r="F29" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
+      <c r="G29" t="b">
+        <v>0</v>
+      </c>
+      <c r="H29" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30" t="s">
         <v>155</v>
       </c>
@@ -7323,39 +7453,48 @@
         <v>-0.1000000000000005</v>
       </c>
       <c r="C30" t="s">
-        <v>165</v>
+        <v>84</v>
       </c>
       <c r="D30" t="s">
-        <v>84</v>
+        <v>526</v>
       </c>
       <c r="E30" t="s">
         <v>137</v>
       </c>
-      <c r="F30" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
+      <c r="G30" t="b">
+        <v>0</v>
+      </c>
+      <c r="H30" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="B31">
         <v>0</v>
       </c>
       <c r="C31" t="s">
-        <v>529</v>
+        <v>466</v>
       </c>
       <c r="D31" t="s">
-        <v>465</v>
+        <v>429</v>
       </c>
       <c r="E31" t="s">
-        <v>542</v>
-      </c>
-      <c r="F31" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
+        <v>434</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31" t="b">
+        <v>0</v>
+      </c>
+      <c r="H31" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" t="s">
         <v>393</v>
       </c>
@@ -7363,19 +7502,22 @@
         <v>28</v>
       </c>
       <c r="C32" t="s">
-        <v>530</v>
+        <v>108</v>
       </c>
       <c r="D32" t="s">
-        <v>108</v>
+        <v>431</v>
       </c>
       <c r="E32" t="s">
         <v>401</v>
       </c>
-      <c r="F32" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6">
+      <c r="G32" t="b">
+        <v>0</v>
+      </c>
+      <c r="H32" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" t="s">
         <v>394</v>
       </c>
@@ -7383,19 +7525,22 @@
         <v>24</v>
       </c>
       <c r="C33" t="s">
-        <v>530</v>
+        <v>108</v>
       </c>
       <c r="D33" t="s">
-        <v>108</v>
+        <v>431</v>
       </c>
       <c r="E33" t="s">
         <v>401</v>
       </c>
-      <c r="F33" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6">
+      <c r="G33" t="b">
+        <v>0</v>
+      </c>
+      <c r="H33" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34" t="s">
         <v>395</v>
       </c>
@@ -7403,19 +7548,22 @@
         <v>0.5283018867924528</v>
       </c>
       <c r="C34" t="s">
-        <v>530</v>
+        <v>108</v>
       </c>
       <c r="D34" t="s">
-        <v>108</v>
+        <v>431</v>
       </c>
       <c r="E34" t="s">
         <v>401</v>
       </c>
-      <c r="F34" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6">
+      <c r="G34" t="b">
+        <v>0</v>
+      </c>
+      <c r="H34" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" t="s">
         <v>396</v>
       </c>
@@ -7423,19 +7571,22 @@
         <v>0.5849056603773585</v>
       </c>
       <c r="C35" t="s">
-        <v>530</v>
+        <v>108</v>
       </c>
       <c r="D35" t="s">
-        <v>108</v>
+        <v>431</v>
       </c>
       <c r="E35" t="s">
         <v>401</v>
       </c>
-      <c r="F35" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6">
+      <c r="G35" t="b">
+        <v>0</v>
+      </c>
+      <c r="H35" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36" t="s">
         <v>397</v>
       </c>
@@ -7443,19 +7594,22 @@
         <v>0.6037735849056604</v>
       </c>
       <c r="C36" t="s">
-        <v>530</v>
+        <v>108</v>
       </c>
       <c r="D36" t="s">
-        <v>108</v>
+        <v>431</v>
       </c>
       <c r="E36" t="s">
         <v>401</v>
       </c>
-      <c r="F36" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6">
+      <c r="G36" t="b">
+        <v>0</v>
+      </c>
+      <c r="H36" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" t="s">
         <v>398</v>
       </c>
@@ -7463,19 +7617,22 @@
         <v>0.660377358490566</v>
       </c>
       <c r="C37" t="s">
-        <v>530</v>
+        <v>108</v>
       </c>
       <c r="D37" t="s">
-        <v>108</v>
+        <v>431</v>
       </c>
       <c r="E37" t="s">
         <v>401</v>
       </c>
-      <c r="F37" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
+      <c r="G37" t="b">
+        <v>0</v>
+      </c>
+      <c r="H37" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" t="s">
         <v>399</v>
       </c>
@@ -7483,19 +7640,22 @@
         <v>7</v>
       </c>
       <c r="C38" t="s">
-        <v>530</v>
+        <v>108</v>
       </c>
       <c r="D38" t="s">
-        <v>108</v>
+        <v>431</v>
       </c>
       <c r="E38" t="s">
         <v>401</v>
       </c>
-      <c r="F38" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
+      <c r="G38" t="b">
+        <v>0</v>
+      </c>
+      <c r="H38" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39" t="s">
         <v>400</v>
       </c>
@@ -7503,800 +7663,998 @@
         <v>5</v>
       </c>
       <c r="C39" t="s">
-        <v>530</v>
+        <v>108</v>
       </c>
       <c r="D39" t="s">
-        <v>108</v>
+        <v>431</v>
       </c>
       <c r="E39" t="s">
         <v>401</v>
       </c>
-      <c r="F39" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
+      <c r="G39" t="b">
+        <v>0</v>
+      </c>
+      <c r="H39" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="B40">
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>531</v>
+        <v>466</v>
       </c>
       <c r="D40" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E40" t="s">
         <v>110</v>
       </c>
-      <c r="F40" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
+      <c r="F40">
+        <v>1</v>
+      </c>
+      <c r="G40" t="b">
+        <v>0</v>
+      </c>
+      <c r="H40" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="B41">
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="D41" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E41" t="s">
         <v>110</v>
       </c>
-      <c r="F41" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41" t="b">
+        <v>0</v>
+      </c>
+      <c r="H41" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="B42">
         <v>0</v>
       </c>
       <c r="C42" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D42" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E42" t="s">
         <v>110</v>
       </c>
-      <c r="F42" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6">
+      <c r="G42" t="b">
+        <v>0</v>
+      </c>
+      <c r="H42" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B43">
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>534</v>
+        <v>466</v>
       </c>
       <c r="D43" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E43" t="s">
         <v>432</v>
       </c>
-      <c r="F43" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6">
+      <c r="F43">
+        <v>1</v>
+      </c>
+      <c r="G43" t="b">
+        <v>0</v>
+      </c>
+      <c r="H43" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="B44">
         <v>1</v>
       </c>
       <c r="C44" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="D44" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E44" t="s">
         <v>432</v>
       </c>
-      <c r="F44" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6">
+      <c r="F44">
+        <v>1</v>
+      </c>
+      <c r="G44" t="b">
+        <v>0</v>
+      </c>
+      <c r="H44" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="B45">
         <v>0</v>
       </c>
       <c r="C45" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D45" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E45" t="s">
         <v>432</v>
       </c>
-      <c r="F45" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6">
+      <c r="G45" t="b">
+        <v>0</v>
+      </c>
+      <c r="H45" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
       <c r="A46" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B46">
         <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>534</v>
+        <v>466</v>
       </c>
       <c r="D46" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E46" t="s">
         <v>432</v>
       </c>
-      <c r="F46" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6">
+      <c r="F46">
+        <v>1</v>
+      </c>
+      <c r="G46" t="b">
+        <v>0</v>
+      </c>
+      <c r="H46" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
       <c r="A47" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="B47">
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="D47" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E47" t="s">
         <v>432</v>
       </c>
-      <c r="F47" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6">
+      <c r="F47">
+        <v>1</v>
+      </c>
+      <c r="G47" t="b">
+        <v>0</v>
+      </c>
+      <c r="H47" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="B48">
         <v>0</v>
       </c>
       <c r="C48" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D48" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E48" t="s">
         <v>432</v>
       </c>
-      <c r="F48" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6">
+      <c r="G48" t="b">
+        <v>0</v>
+      </c>
+      <c r="H48" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B49">
         <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>534</v>
+        <v>466</v>
       </c>
       <c r="D49" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E49" t="s">
         <v>432</v>
       </c>
-      <c r="F49" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6">
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49" t="b">
+        <v>0</v>
+      </c>
+      <c r="H49" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="B50">
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="D50" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E50" t="s">
         <v>432</v>
       </c>
-      <c r="F50" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6">
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50" t="b">
+        <v>0</v>
+      </c>
+      <c r="H50" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="B51">
         <v>0</v>
       </c>
       <c r="C51" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D51" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E51" t="s">
         <v>432</v>
       </c>
-      <c r="F51" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6">
+      <c r="G51" t="b">
+        <v>0</v>
+      </c>
+      <c r="H51" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B52">
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>534</v>
+        <v>466</v>
       </c>
       <c r="D52" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E52" t="s">
         <v>432</v>
       </c>
-      <c r="F52" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6">
+      <c r="F52">
+        <v>1</v>
+      </c>
+      <c r="G52" t="b">
+        <v>0</v>
+      </c>
+      <c r="H52" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="B53">
         <v>1</v>
       </c>
       <c r="C53" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="D53" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E53" t="s">
         <v>432</v>
       </c>
-      <c r="F53" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6">
+      <c r="F53">
+        <v>1</v>
+      </c>
+      <c r="G53" t="b">
+        <v>0</v>
+      </c>
+      <c r="H53" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
       <c r="A54" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="B54">
         <v>0</v>
       </c>
       <c r="C54" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D54" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E54" t="s">
         <v>432</v>
       </c>
-      <c r="F54" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6">
+      <c r="G54" t="b">
+        <v>0</v>
+      </c>
+      <c r="H54" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
       <c r="A55" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B55">
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>534</v>
+        <v>466</v>
       </c>
       <c r="D55" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E55" t="s">
         <v>432</v>
       </c>
-      <c r="F55" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6">
+      <c r="F55">
+        <v>1</v>
+      </c>
+      <c r="G55" t="b">
+        <v>0</v>
+      </c>
+      <c r="H55" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
       <c r="A56" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="B56">
         <v>1</v>
       </c>
       <c r="C56" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="D56" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E56" t="s">
         <v>432</v>
       </c>
-      <c r="F56" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6">
+      <c r="F56">
+        <v>1</v>
+      </c>
+      <c r="G56" t="b">
+        <v>0</v>
+      </c>
+      <c r="H56" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
       <c r="A57" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="B57">
         <v>0</v>
       </c>
       <c r="C57" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D57" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E57" t="s">
         <v>432</v>
       </c>
-      <c r="F57" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6">
+      <c r="G57" t="b">
+        <v>0</v>
+      </c>
+      <c r="H57" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
       <c r="A58" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B58">
         <v>1</v>
       </c>
       <c r="C58" t="s">
-        <v>534</v>
+        <v>466</v>
       </c>
       <c r="D58" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E58" t="s">
         <v>432</v>
       </c>
-      <c r="F58" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6">
+      <c r="F58">
+        <v>1</v>
+      </c>
+      <c r="G58" t="b">
+        <v>0</v>
+      </c>
+      <c r="H58" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
       <c r="A59" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="B59">
         <v>1</v>
       </c>
       <c r="C59" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="D59" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E59" t="s">
         <v>432</v>
       </c>
-      <c r="F59" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6">
+      <c r="F59">
+        <v>1</v>
+      </c>
+      <c r="G59" t="b">
+        <v>0</v>
+      </c>
+      <c r="H59" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
       <c r="A60" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="B60">
         <v>0</v>
       </c>
       <c r="C60" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D60" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E60" t="s">
         <v>432</v>
       </c>
-      <c r="F60" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6">
+      <c r="G60" t="b">
+        <v>0</v>
+      </c>
+      <c r="H60" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
       <c r="A61" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B61">
         <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>534</v>
+        <v>466</v>
       </c>
       <c r="D61" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E61" t="s">
         <v>432</v>
       </c>
-      <c r="F61" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6">
+      <c r="F61">
+        <v>1</v>
+      </c>
+      <c r="G61" t="b">
+        <v>0</v>
+      </c>
+      <c r="H61" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
       <c r="A62" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="B62">
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="D62" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E62" t="s">
         <v>432</v>
       </c>
-      <c r="F62" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6">
+      <c r="F62">
+        <v>1</v>
+      </c>
+      <c r="G62" t="b">
+        <v>0</v>
+      </c>
+      <c r="H62" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
       <c r="A63" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="B63">
         <v>0</v>
       </c>
       <c r="C63" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D63" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E63" t="s">
         <v>432</v>
       </c>
-      <c r="F63" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6">
+      <c r="G63" t="b">
+        <v>0</v>
+      </c>
+      <c r="H63" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
       <c r="A64" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="B64">
         <v>1</v>
       </c>
       <c r="C64" t="s">
-        <v>535</v>
+        <v>466</v>
       </c>
       <c r="D64" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E64" t="s">
         <v>390</v>
       </c>
-      <c r="F64" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6">
+      <c r="F64">
+        <v>1</v>
+      </c>
+      <c r="G64" t="b">
+        <v>0</v>
+      </c>
+      <c r="H64" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
       <c r="A65" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="B65">
         <v>1</v>
       </c>
       <c r="C65" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="D65" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E65" t="s">
         <v>390</v>
       </c>
-      <c r="F65" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6">
+      <c r="F65">
+        <v>1</v>
+      </c>
+      <c r="G65" t="b">
+        <v>0</v>
+      </c>
+      <c r="H65" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
       <c r="A66" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="B66">
         <v>0</v>
       </c>
       <c r="C66" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D66" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E66" t="s">
         <v>390</v>
       </c>
-      <c r="F66" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6">
+      <c r="G66" t="b">
+        <v>0</v>
+      </c>
+      <c r="H66" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
       <c r="A67" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="B67">
         <v>0.9423076923076923</v>
       </c>
       <c r="C67" t="s">
-        <v>536</v>
+        <v>466</v>
       </c>
       <c r="D67" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E67" t="s">
         <v>433</v>
       </c>
-      <c r="F67" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6">
+      <c r="F67">
+        <v>0.9423076923076923</v>
+      </c>
+      <c r="G67" t="b">
+        <v>0</v>
+      </c>
+      <c r="H67" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
       <c r="A68" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="B68">
         <v>0.9876091402011571</v>
       </c>
       <c r="C68" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="D68" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E68" t="s">
         <v>433</v>
       </c>
-      <c r="F68" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6">
+      <c r="F68">
+        <v>0.9876091402011571</v>
+      </c>
+      <c r="G68" t="b">
+        <v>0</v>
+      </c>
+      <c r="H68" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
       <c r="A69" t="s">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="B69">
         <v>0</v>
       </c>
       <c r="C69" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D69" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E69" t="s">
         <v>433</v>
       </c>
-      <c r="F69" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6">
+      <c r="G69" t="b">
+        <v>0</v>
+      </c>
+      <c r="H69" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
       <c r="A70" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B70">
         <v>0</v>
       </c>
       <c r="C70" t="s">
-        <v>537</v>
+        <v>466</v>
       </c>
       <c r="D70" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E70" t="s">
         <v>434</v>
       </c>
-      <c r="F70" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6">
+      <c r="F70">
+        <v>0</v>
+      </c>
+      <c r="G70" t="b">
+        <v>0</v>
+      </c>
+      <c r="H70" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
       <c r="A71" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="B71">
         <v>0</v>
       </c>
       <c r="C71" t="s">
-        <v>532</v>
+        <v>466</v>
       </c>
       <c r="D71" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E71" t="s">
         <v>434</v>
       </c>
-      <c r="F71" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6">
+      <c r="F71">
+        <v>0</v>
+      </c>
+      <c r="G71" t="b">
+        <v>0</v>
+      </c>
+      <c r="H71" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
       <c r="A72" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="B72">
         <v>0</v>
       </c>
       <c r="C72" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D72" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E72" t="s">
         <v>434</v>
       </c>
-      <c r="F72" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6">
+      <c r="G72" t="b">
+        <v>0</v>
+      </c>
+      <c r="H72" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
       <c r="A73" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="B73">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="C73" t="s">
-        <v>538</v>
+        <v>466</v>
       </c>
       <c r="D73" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E73" t="s">
         <v>435</v>
       </c>
-      <c r="F73" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6">
+      <c r="F73">
+        <v>0.9</v>
+      </c>
+      <c r="G73" t="b">
+        <v>0</v>
+      </c>
+      <c r="H73" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8">
       <c r="A74" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
       <c r="B74">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="C74" t="s">
-        <v>539</v>
+        <v>466</v>
       </c>
       <c r="D74" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E74" t="s">
         <v>435</v>
       </c>
-      <c r="F74" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6">
+      <c r="F74">
+        <v>0.9</v>
+      </c>
+      <c r="G74" t="b">
+        <v>0</v>
+      </c>
+      <c r="H74" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
       <c r="A75" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
       <c r="B75">
         <v>0</v>
       </c>
       <c r="C75" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D75" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E75" t="s">
         <v>435</v>
       </c>
-      <c r="F75" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6">
+      <c r="G75" t="b">
+        <v>0</v>
+      </c>
+      <c r="H75" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
       <c r="A76" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
       <c r="B76">
         <v>0.5408163265306123</v>
       </c>
       <c r="C76" t="s">
-        <v>540</v>
+        <v>466</v>
       </c>
       <c r="D76" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E76" t="s">
         <v>401</v>
       </c>
-      <c r="F76" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6">
+      <c r="F76">
+        <v>0.5408163265306123</v>
+      </c>
+      <c r="G76" t="b">
+        <v>0</v>
+      </c>
+      <c r="H76" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
       <c r="A77" t="s">
-        <v>518</v>
+        <v>523</v>
       </c>
       <c r="B77">
         <v>0.4689190577470169</v>
       </c>
       <c r="C77" t="s">
-        <v>541</v>
+        <v>466</v>
       </c>
       <c r="D77" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E77" t="s">
         <v>401</v>
       </c>
-      <c r="F77" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6">
+      <c r="F77">
+        <v>0.4689190577470169</v>
+      </c>
+      <c r="G77" t="b">
+        <v>0</v>
+      </c>
+      <c r="H77" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
       <c r="A78" t="s">
-        <v>519</v>
+        <v>524</v>
       </c>
       <c r="B78">
         <v>0</v>
       </c>
       <c r="C78" t="s">
-        <v>533</v>
+        <v>466</v>
       </c>
       <c r="D78" t="s">
-        <v>465</v>
+        <v>527</v>
       </c>
       <c r="E78" t="s">
         <v>401</v>
       </c>
-      <c r="F78" t="b">
-        <v>0</v>
+      <c r="G78" t="b">
+        <v>0</v>
+      </c>
+      <c r="H78" t="s">
+        <v>541</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F78"/>
+  <autoFilter ref="A1:H78"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -8314,7 +8672,7 @@
         <v>408</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>543</v>
+        <v>556</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -8331,7 +8689,7 @@
         <v>110</v>
       </c>
       <c r="B2" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="C2" t="s">
         <v>109</v>
@@ -8340,7 +8698,7 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -8348,7 +8706,7 @@
         <v>432</v>
       </c>
       <c r="B3" t="s">
-        <v>546</v>
+        <v>559</v>
       </c>
       <c r="C3" t="s">
         <v>123</v>
@@ -8357,7 +8715,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -8365,7 +8723,7 @@
         <v>432</v>
       </c>
       <c r="B4" t="s">
-        <v>546</v>
+        <v>559</v>
       </c>
       <c r="C4" t="s">
         <v>124</v>
@@ -8374,7 +8732,7 @@
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -8382,7 +8740,7 @@
         <v>432</v>
       </c>
       <c r="B5" t="s">
-        <v>546</v>
+        <v>559</v>
       </c>
       <c r="C5" t="s">
         <v>125</v>
@@ -8391,7 +8749,7 @@
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -8399,7 +8757,7 @@
         <v>432</v>
       </c>
       <c r="B6" t="s">
-        <v>546</v>
+        <v>559</v>
       </c>
       <c r="C6" t="s">
         <v>126</v>
@@ -8408,7 +8766,7 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -8416,7 +8774,7 @@
         <v>432</v>
       </c>
       <c r="B7" t="s">
-        <v>546</v>
+        <v>559</v>
       </c>
       <c r="C7" t="s">
         <v>127</v>
@@ -8425,7 +8783,7 @@
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -8433,7 +8791,7 @@
         <v>432</v>
       </c>
       <c r="B8" t="s">
-        <v>546</v>
+        <v>559</v>
       </c>
       <c r="C8" t="s">
         <v>128</v>
@@ -8442,7 +8800,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -8450,7 +8808,7 @@
         <v>432</v>
       </c>
       <c r="B9" t="s">
-        <v>546</v>
+        <v>559</v>
       </c>
       <c r="C9" t="s">
         <v>129</v>
@@ -8459,7 +8817,7 @@
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -8476,7 +8834,7 @@
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -8484,33 +8842,33 @@
         <v>434</v>
       </c>
       <c r="B11" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C11" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D11" t="b">
         <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>544</v>
+        <v>557</v>
       </c>
       <c r="B12" t="s">
-        <v>547</v>
+        <v>560</v>
       </c>
       <c r="C12" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D12" t="b">
         <v>1</v>
       </c>
       <c r="E12" t="s">
-        <v>548</v>
+        <v>561</v>
       </c>
     </row>
   </sheetData>
@@ -14260,23 +14618,8 @@
       <c r="C10">
         <v>0.03183849</v>
       </c>
-      <c r="D10">
-        <v>365.76001</v>
-      </c>
-      <c r="E10">
-        <v>-3.50998</v>
-      </c>
-      <c r="F10">
-        <v>-0.95051842</v>
-      </c>
-      <c r="J10" t="s">
-        <v>410</v>
-      </c>
-      <c r="K10">
-        <v>1780666200</v>
-      </c>
       <c r="L10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -14289,23 +14632,8 @@
       <c r="C11">
         <v>0.0314861</v>
       </c>
-      <c r="D11">
-        <v>385.73001</v>
-      </c>
-      <c r="E11">
-        <v>-33.17999</v>
-      </c>
-      <c r="F11">
-        <v>-7.92055</v>
-      </c>
-      <c r="J11" t="s">
-        <v>410</v>
-      </c>
-      <c r="K11">
-        <v>1780666200</v>
-      </c>
       <c r="L11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -14703,7 +15031,7 @@
         <v>0</v>
       </c>
       <c r="O2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -14741,7 +15069,7 @@
         <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -14779,7 +15107,7 @@
         <v>0</v>
       </c>
       <c r="O4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -14817,7 +15145,7 @@
         <v>0</v>
       </c>
       <c r="O5" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -14855,7 +15183,7 @@
         <v>0</v>
       </c>
       <c r="O6" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -14893,7 +15221,7 @@
         <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -14931,7 +15259,7 @@
         <v>0</v>
       </c>
       <c r="O8" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -14969,7 +15297,7 @@
         <v>0</v>
       </c>
       <c r="O9" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -15007,7 +15335,7 @@
         <v>0</v>
       </c>
       <c r="O10" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -15048,7 +15376,7 @@
         <v>0</v>
       </c>
       <c r="O11" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -15089,7 +15417,7 @@
         <v>0</v>
       </c>
       <c r="O12" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -15106,10 +15434,16 @@
         <v>20</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>0.9</v>
+      </c>
+      <c r="G13" t="s">
+        <v>438</v>
+      </c>
+      <c r="H13" t="s">
+        <v>438</v>
       </c>
       <c r="I13" t="b">
         <v>0</v>
@@ -15130,7 +15464,7 @@
         <v>410</v>
       </c>
       <c r="O13" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -15153,10 +15487,10 @@
         <v>0.4689190577470169</v>
       </c>
       <c r="G14" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="H14" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="I14" t="b">
         <v>0</v>
@@ -15174,10 +15508,10 @@
         <v>0</v>
       </c>
       <c r="N14" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="O14" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update daily Nasdaq-100 QQQ tracker outputs
</commit_message>
<xml_diff>
--- a/reports/archive/2026-06-06/nasdaq100_qqq_daily_tracker_2026-06-06.xlsx
+++ b/reports/archive/2026-06-06/nasdaq100_qqq_daily_tracker_2026-06-06.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3108" uniqueCount="742">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3110" uniqueCount="742">
   <si>
     <t>date</t>
   </si>
@@ -1936,7 +1936,7 @@
     <t>20/20 top20 quotes available; 10/10 top10 quotes available</t>
   </si>
   <si>
-    <t>98/98 symbols with history coverage; 20/98 history symbols with Twelve Data quote overlay</t>
+    <t>97/98 symbols with history coverage; 19/97 history symbols with Twelve Data quote overlay; coverage insufficient for top-weight symbols</t>
   </si>
   <si>
     <t>run_date</t>
@@ -2194,7 +2194,7 @@
     <t>latest FRED observation value</t>
   </si>
   <si>
-    <t>breadth metric; denominator=98</t>
+    <t>breadth metric; denominator=97</t>
   </si>
   <si>
     <t>symbol coverage; ok=True; rows=260; message=QQQ cache ready</t>
@@ -2242,7 +2242,7 @@
     <t>weight coverage; rate_limited=False; fallback_provider=quote_cache</t>
   </si>
   <si>
-    <t>symbol coverage; ok=True; rows=8; message=98/98 symbols with history coverage; 20/98 history symbols with Twelve Data quote overlay</t>
+    <t>symbol coverage; ok=True; rows=8; message=97/98 symbols with history coverage; 19/97 history symbols with Twelve Data quote overlay; coverage insufficient for top-weight symbols</t>
   </si>
   <si>
     <t>weight coverage; rate_limited=False; fallback_provider=twelve_data_quote</t>
@@ -2266,7 +2266,7 @@
     <t>98 symbols</t>
   </si>
   <si>
-    <t>98/98 symbols loaded from local cache/raw seed</t>
+    <t>97/98 symbols loaded from local cache/raw seed</t>
   </si>
 </sst>
 </file>
@@ -7825,13 +7825,13 @@
         <v>609.65</v>
       </c>
       <c r="G179">
-        <v>608.8911435241999</v>
+        <v>609.65</v>
       </c>
       <c r="H179" s="1">
         <v>78019338</v>
       </c>
       <c r="I179" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="180" spans="1:9">
@@ -9252,7 +9252,7 @@
         <v>37138511</v>
       </c>
       <c r="I228" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="229" spans="1:9">
@@ -9774,7 +9774,7 @@
         <v>33327545</v>
       </c>
       <c r="I246" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="247" spans="1:9">
@@ -10771,10 +10771,16 @@
         <v>8</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>0.9897959183673469</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>0.9146145309607144</v>
+      </c>
+      <c r="G13" t="s">
+        <v>333</v>
+      </c>
+      <c r="H13" t="s">
+        <v>333</v>
       </c>
       <c r="I13" t="b">
         <v>0</v>
@@ -10786,7 +10792,7 @@
         <v>0</v>
       </c>
       <c r="L13">
-        <v>28168</v>
+        <v>27880</v>
       </c>
       <c r="M13">
         <v>0</v>
@@ -10795,10 +10801,10 @@
         <v>618</v>
       </c>
       <c r="O13">
-        <v>1</v>
+        <v>0.9897959183673469</v>
       </c>
       <c r="P13">
-        <v>0.2040816326530612</v>
+        <v>0.1958762886597938</v>
       </c>
       <c r="T13" t="s">
         <v>577</v>
@@ -11496,7 +11502,7 @@
         <v>680</v>
       </c>
       <c r="B9">
-        <v>621.0349008439025</v>
+        <v>621.0386951262815</v>
       </c>
       <c r="C9" t="s">
         <v>268</v>
@@ -12025,7 +12031,7 @@
         <v>556</v>
       </c>
       <c r="B32">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C32" t="s">
         <v>268</v>
@@ -12048,7 +12054,7 @@
         <v>557</v>
       </c>
       <c r="B33">
-        <v>0.4285714285714285</v>
+        <v>0.4329896907216495</v>
       </c>
       <c r="C33" t="s">
         <v>268</v>
@@ -12071,7 +12077,7 @@
         <v>558</v>
       </c>
       <c r="B34">
-        <v>0.5306122448979592</v>
+        <v>0.5360824742268041</v>
       </c>
       <c r="C34" t="s">
         <v>268</v>
@@ -12094,7 +12100,7 @@
         <v>559</v>
       </c>
       <c r="B35">
-        <v>0.5714285714285714</v>
+        <v>0.5670103092783505</v>
       </c>
       <c r="C35" t="s">
         <v>268</v>
@@ -12117,7 +12123,7 @@
         <v>560</v>
       </c>
       <c r="B36">
-        <v>0.5918367346938775</v>
+        <v>0.5876288659793815</v>
       </c>
       <c r="C36" t="s">
         <v>268</v>
@@ -12163,7 +12169,7 @@
         <v>562</v>
       </c>
       <c r="B38">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C38" t="s">
         <v>268</v>
@@ -13011,7 +13017,7 @@
         <v>702</v>
       </c>
       <c r="B72">
-        <v>1</v>
+        <v>0.9897959183673469</v>
       </c>
       <c r="C72" t="s">
         <v>648</v>
@@ -13023,7 +13029,7 @@
         <v>563</v>
       </c>
       <c r="F72">
-        <v>1</v>
+        <v>0.9897959183673469</v>
       </c>
       <c r="G72" t="b">
         <v>0</v>
@@ -13037,7 +13043,7 @@
         <v>703</v>
       </c>
       <c r="B73">
-        <v>1</v>
+        <v>0.9146145309607144</v>
       </c>
       <c r="C73" t="s">
         <v>648</v>
@@ -13049,7 +13055,7 @@
         <v>563</v>
       </c>
       <c r="F73">
-        <v>1</v>
+        <v>0.9146145309607144</v>
       </c>
       <c r="G73" t="b">
         <v>0</v>
@@ -13369,7 +13375,7 @@
         <v>667.8092</v>
       </c>
       <c r="K2">
-        <v>621.0349008439025</v>
+        <v>621.0386951262815</v>
       </c>
     </row>
   </sheetData>
@@ -18580,7 +18586,7 @@
         <v>42</v>
       </c>
       <c r="C2">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D2" t="s">
         <v>268</v>
@@ -18597,10 +18603,10 @@
         <v>556</v>
       </c>
       <c r="B3">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C3">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
         <v>268</v>
@@ -18617,10 +18623,10 @@
         <v>557</v>
       </c>
       <c r="B4">
-        <v>0.4285714285714285</v>
+        <v>0.4329896907216495</v>
       </c>
       <c r="C4">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
         <v>268</v>
@@ -18637,10 +18643,10 @@
         <v>558</v>
       </c>
       <c r="B5">
-        <v>0.5306122448979592</v>
+        <v>0.5360824742268041</v>
       </c>
       <c r="C5">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D5" t="s">
         <v>268</v>
@@ -18657,10 +18663,10 @@
         <v>559</v>
       </c>
       <c r="B6">
-        <v>0.5714285714285714</v>
+        <v>0.5670103092783505</v>
       </c>
       <c r="C6">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D6" t="s">
         <v>268</v>
@@ -18677,10 +18683,10 @@
         <v>560</v>
       </c>
       <c r="B7">
-        <v>0.5918367346938775</v>
+        <v>0.5876288659793815</v>
       </c>
       <c r="C7">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D7" t="s">
         <v>268</v>
@@ -18700,7 +18706,7 @@
         <v>9</v>
       </c>
       <c r="C8">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D8" t="s">
         <v>268</v>
@@ -18717,10 +18723,10 @@
         <v>562</v>
       </c>
       <c r="B9">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D9" t="s">
         <v>268</v>

</xml_diff>